<commit_message>
Regenera artefactos BAU y habilita del_files en Config_MOMF_T1_AB
- Actualiza inputs/outputs del escenario BAU tras correr el pipeline
  completo: A1_Outputs_BAU/A-O_*.xlsx, A2_Extra_Inputs/*.xlsx,
  A2_Output_Params/BAU/*.csv, Executables/BAU_0/BAU_0_Input.csv y los
  Pre_processed_BAU_0*.txt encadenados (NoStorage, OpenBCK,
  RMCarefulXLSX) más sus warnings, cplex.log y output.csv.
- Elimina BAU_0.txt y Executables/BAU_0/Outputs/*.csv: con
  del_files: True la corrida los limpia al final, así que no deben
  quedar versionados.
- Config_MOMF_T1_AB.yaml: del_files False → True.
</commit_message>
<xml_diff>
--- a/t1_confection/A2_Extra_Inputs/A-Xtra_Storage.xlsx
+++ b/t1_confection/A2_Extra_Inputs/A-Xtra_Storage.xlsx
@@ -2562,11 +2562,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ResidualStorageCapacity</t>
+          <t>CapitalCostStorage</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2575,88 +2575,88 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="J10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="K10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="L10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="M10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="N10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="O10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="P10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="R10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="S10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="T10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="U10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="V10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="W10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="X10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AI10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.036</v>
+        <v>52694.44444444445</v>
       </c>
     </row>
     <row r="11">
@@ -2674,11 +2674,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CapitalCostStorage</t>
+          <t>ResidualStorageCapacity</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2687,88 +2687,88 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="J11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="K11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="L11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="M11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="N11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="O11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="P11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="Q11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="R11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="S11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="T11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="U11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="V11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="W11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="X11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="Y11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="Z11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AA11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AB11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AC11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AD11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AE11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AF11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AG11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AH11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AI11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
       <c r="AJ11" t="n">
-        <v>52694.44444444445</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="12">
@@ -3682,101 +3682,101 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ResidualStorageCapacity</t>
+          <t>CapitalCostStorage</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>EMPTY</t>
+          <t>User defined</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="J20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="K20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="L20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="M20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="N20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="O20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="P20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="Q20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="R20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="S20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="T20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="U20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="V20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="W20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="X20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="Y20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="Z20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AA20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AB20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AC20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AD20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AE20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AF20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AG20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AH20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AI20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
       <c r="AJ20" t="n">
-        <v/>
+        <v>52694.44444444445</v>
       </c>
     </row>
     <row r="21">
@@ -3794,101 +3794,101 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CapitalCostStorage</t>
+          <t>ResidualStorageCapacity</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>User defined</t>
+          <t>EMPTY</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="J21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="K21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="L21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="M21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="N21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="O21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="P21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="Q21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="R21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="S21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="T21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="U21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="V21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="W21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="X21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="Y21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="Z21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AA21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AB21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AC21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AD21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AE21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AF21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AG21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AH21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AI21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
       <c r="AJ21" t="n">
-        <v>52694.44444444445</v>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -4802,11 +4802,11 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ResidualStorageCapacity</t>
+          <t>CapitalCostStorage</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -4815,88 +4815,88 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="J30" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="K30" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="L30" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="M30" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="N30" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="O30" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="P30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="R30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="S30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="T30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="U30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="V30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="W30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="X30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="Z30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AA30" t="n">
-        <v>0.00156</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AB30" t="n">
-        <v>0.00153</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AC30" t="n">
-        <v>0.00153</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AD30" t="n">
-        <v>0.00153</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AE30" t="n">
-        <v>0.00153</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AF30" t="n">
-        <v>0.00153</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AG30" t="n">
-        <v>0.00148</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AH30" t="n">
-        <v>0.00148</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AI30" t="n">
-        <v>0.00148</v>
+        <v>67291.66666666667</v>
       </c>
       <c r="AJ30" t="n">
-        <v>0.00148</v>
+        <v>67291.66666666667</v>
       </c>
     </row>
     <row r="31">
@@ -4914,11 +4914,11 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CapitalCostStorage</t>
+          <t>ResidualStorageCapacity</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -4927,88 +4927,88 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>67291.66666666667</v>
+        <v>9.000000000000001e-05</v>
       </c>
       <c r="J31" t="n">
-        <v>67291.66666666667</v>
+        <v>9.000000000000001e-05</v>
       </c>
       <c r="K31" t="n">
-        <v>67291.66666666667</v>
+        <v>9.000000000000001e-05</v>
       </c>
       <c r="L31" t="n">
-        <v>67291.66666666667</v>
+        <v>9.000000000000001e-05</v>
       </c>
       <c r="M31" t="n">
-        <v>67291.66666666667</v>
+        <v>9.000000000000001e-05</v>
       </c>
       <c r="N31" t="n">
-        <v>67291.66666666667</v>
+        <v>9.000000000000001e-05</v>
       </c>
       <c r="O31" t="n">
-        <v>67291.66666666667</v>
+        <v>9.000000000000001e-05</v>
       </c>
       <c r="P31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="Q31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="R31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="S31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="T31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="U31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="V31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="W31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="X31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="Y31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="Z31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="AA31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00156</v>
       </c>
       <c r="AB31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00153</v>
       </c>
       <c r="AC31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00153</v>
       </c>
       <c r="AD31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00153</v>
       </c>
       <c r="AE31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00153</v>
       </c>
       <c r="AF31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00153</v>
       </c>
       <c r="AG31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00148</v>
       </c>
       <c r="AH31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00148</v>
       </c>
       <c r="AI31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00148</v>
       </c>
       <c r="AJ31" t="n">
-        <v>67291.66666666667</v>
+        <v>0.00148</v>
       </c>
     </row>
     <row r="32">

</xml_diff>